<commit_message>
auto: 작업 자동 저장 2026-09-10 09:49
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/results/전달함_팀장님/CI_arm실험세트_집계.xlsx
+++ b/eval-runner/orchestrator/results/전달함_팀장님/CI_arm실험세트_집계.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arm 비교" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="F 확인" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1185,4 +1186,341 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>확인 1벌 F(512·off·폭100) — D에서 정렬만 뺀 것 · 채택 판정 (비E형 447 · 건수만 · 2026-09-10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>arm</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>top5</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>top1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>앵커 120</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>표 235</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>문장 127</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FAQ 85</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>후보 안 21 회수</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>밖 119→top5</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>A 대비 신규</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>A 대비 이탈</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>이탈 중 표</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>v3.1</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>293</v>
+      </c>
+      <c r="C4" t="n">
+        <v>216</v>
+      </c>
+      <c r="D4" t="n">
+        <v>83</v>
+      </c>
+      <c r="E4" t="n">
+        <v>135</v>
+      </c>
+      <c r="F4" t="n">
+        <v>96</v>
+      </c>
+      <c r="G4" t="n">
+        <v>62</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>294</v>
+      </c>
+      <c r="C5" t="n">
+        <v>217</v>
+      </c>
+      <c r="D5" t="n">
+        <v>83</v>
+      </c>
+      <c r="E5" t="n">
+        <v>135</v>
+      </c>
+      <c r="F5" t="n">
+        <v>96</v>
+      </c>
+      <c r="G5" t="n">
+        <v>63</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>299</v>
+      </c>
+      <c r="C6" t="n">
+        <v>226</v>
+      </c>
+      <c r="D6" t="n">
+        <v>85</v>
+      </c>
+      <c r="E6" t="n">
+        <v>142</v>
+      </c>
+      <c r="F6" t="n">
+        <v>97</v>
+      </c>
+      <c r="G6" t="n">
+        <v>60</v>
+      </c>
+      <c r="H6" t="n">
+        <v>11</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>18</v>
+      </c>
+      <c r="K6" t="n">
+        <v>13</v>
+      </c>
+      <c r="L6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>308</v>
+      </c>
+      <c r="C7" t="n">
+        <v>227</v>
+      </c>
+      <c r="D7" t="n">
+        <v>82</v>
+      </c>
+      <c r="E7" t="n">
+        <v>147</v>
+      </c>
+      <c r="F7" t="n">
+        <v>96</v>
+      </c>
+      <c r="G7" t="n">
+        <v>65</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10</v>
+      </c>
+      <c r="I7" t="n">
+        <v>13</v>
+      </c>
+      <c r="J7" t="n">
+        <v>31</v>
+      </c>
+      <c r="K7" t="n">
+        <v>17</v>
+      </c>
+      <c r="L7" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>310</v>
+      </c>
+      <c r="C8" t="n">
+        <v>230</v>
+      </c>
+      <c r="D8" t="n">
+        <v>87</v>
+      </c>
+      <c r="E8" t="n">
+        <v>149</v>
+      </c>
+      <c r="F8" t="n">
+        <v>99</v>
+      </c>
+      <c r="G8" t="n">
+        <v>62</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10</v>
+      </c>
+      <c r="I8" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" t="n">
+        <v>29</v>
+      </c>
+      <c r="K8" t="n">
+        <v>13</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F↔D top5 판정 바뀐 문항</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>F만 11 · D만 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F 창 재판정</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>적중 290 중 창 안 271 (93%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>속도 P50</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>search 997ms · rerank 396ms · P95 search 1,490ms (동시 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>■ 판정</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>F 채택 → 새 기준선 봉인: top5 310 · top1 230 · 앵커 87 · 표 149 · 문장 99 · FAQ 62 · 미적중 잔여 137(표 86)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>